<commit_message>
Update forecast evaluation for inflation
</commit_message>
<xml_diff>
--- a/IaR_GaR_April_2026/Outputs/forecast_evaluation/comparison_fcst_eval_inflation.xlsx
+++ b/IaR_GaR_April_2026/Outputs/forecast_evaluation/comparison_fcst_eval_inflation.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -21,13 +21,14 @@
     <sheet name="CRPS_mean" sheetId="13" r:id="rId15"/>
     <sheet name="wCRPS_left_mean" sheetId="14" r:id="rId16"/>
     <sheet name="wCRPS_right_mean" sheetId="15" r:id="rId17"/>
+    <sheet name="GMM_summary" sheetId="16" r:id="rId18"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="908" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="71">
   <si>
     <t>horizon</t>
   </si>
@@ -42,12 +43,210 @@
   </si>
   <si>
     <t>qr_sp</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>horizon</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>fanchart</t>
+  </si>
+  <si>
+    <t>qr</t>
+  </si>
+  <si>
+    <t>bvar</t>
+  </si>
+  <si>
+    <t>GMM_KS_std_bonf_w_wi_1</t>
+  </si>
+  <si>
+    <t>GMM_KS_std_bonf_w_wi_2</t>
+  </si>
+  <si>
+    <t>GMM_KS_std_bonf_w_wi_3</t>
+  </si>
+  <si>
+    <t>GMM_CVM_std_bonf_w_wi_1</t>
+  </si>
+  <si>
+    <t>GMM_CVM_std_bonf_w_wi_2</t>
+  </si>
+  <si>
+    <t>GMM_CVM_std_bonf_w_wi_3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -90,25 +289,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="13.453125" customWidth="true"/>
-    <col min="3" max="3" width="13.453125" customWidth="true"/>
-    <col min="4" max="4" width="13.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="13.7109375" customWidth="true"/>
+    <col min="3" max="3" width="13.7109375" customWidth="true"/>
+    <col min="4" max="4" width="13.7109375" customWidth="true"/>
     <col min="5" max="5" width="13.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -122,10 +321,10 @@
         <v>0.18317428429326366</v>
       </c>
       <c r="C2" s="0">
-        <v>0.10519737041931522</v>
+        <v>0.080225496131627827</v>
       </c>
       <c r="D2" s="0">
-        <v>0.074038235294117627</v>
+        <v>0.12023728236014997</v>
       </c>
       <c r="E2" s="0">
         <v>0.12023728236014997</v>
@@ -139,10 +338,10 @@
         <v>0.14288461772367245</v>
       </c>
       <c r="C3" s="0">
-        <v>0.069663526789969593</v>
+        <v>0.1864492194549347</v>
       </c>
       <c r="D3" s="0">
-        <v>0.085739215686274517</v>
+        <v>0.055711349230834512</v>
       </c>
       <c r="E3" s="0">
         <v>0.055711349230834512</v>
@@ -156,10 +355,10 @@
         <v>0.098333723943279855</v>
       </c>
       <c r="C4" s="0">
-        <v>0.10710666983691849</v>
+        <v>0.22490102341226681</v>
       </c>
       <c r="D4" s="0">
-        <v>0.14262058823529411</v>
+        <v>0.086431676384817635</v>
       </c>
       <c r="E4" s="0">
         <v>0.086431676384817635</v>
@@ -173,10 +372,10 @@
         <v>0.088638721022962885</v>
       </c>
       <c r="C5" s="0">
-        <v>0.16807284481898285</v>
+        <v>0.2187198091697134</v>
       </c>
       <c r="D5" s="0">
-        <v>0.16046764705882344</v>
+        <v>0.15555451018106997</v>
       </c>
       <c r="E5" s="0">
         <v>0.15555451018106997</v>
@@ -190,10 +389,10 @@
         <v>0.12425732188398642</v>
       </c>
       <c r="C6" s="0">
-        <v>0.18579978257627727</v>
+        <v>0.21744566305748025</v>
       </c>
       <c r="D6" s="0">
-        <v>0.17858627450980391</v>
+        <v>0.17404337893212718</v>
       </c>
       <c r="E6" s="0">
         <v>0.17404337893212718</v>
@@ -207,10 +406,10 @@
         <v>0.14898862180387296</v>
       </c>
       <c r="C7" s="0">
-        <v>0.19802367922709757</v>
+        <v>0.20501435224460074</v>
       </c>
       <c r="D7" s="0">
-        <v>0.21008627450980388</v>
+        <v>0.16242062143239128</v>
       </c>
       <c r="E7" s="0">
         <v>0.16242062143239128</v>
@@ -224,10 +423,10 @@
         <v>0.14741208004070727</v>
       </c>
       <c r="C8" s="0">
-        <v>0.20333624896164837</v>
+        <v>0.18851936790176671</v>
       </c>
       <c r="D8" s="0">
-        <v>0.21530980392156865</v>
+        <v>0.14562013494340337</v>
       </c>
       <c r="E8" s="0">
         <v>0.14562013494340337</v>
@@ -241,10 +440,10 @@
         <v>0.12908885436803441</v>
       </c>
       <c r="C9" s="0">
-        <v>0.17819265761609593</v>
+        <v>0.27080028618429536</v>
       </c>
       <c r="D9" s="0">
-        <v>0.17853627450980392</v>
+        <v>0.12458385872065492</v>
       </c>
       <c r="E9" s="0">
         <v>0.12458385872065492</v>
@@ -258,10 +457,10 @@
         <v>0.12586259609857597</v>
       </c>
       <c r="C10" s="0">
-        <v>0.26846878034935717</v>
+        <v>0.29130891982510548</v>
       </c>
       <c r="D10" s="0">
-        <v>0.25426764705882343</v>
+        <v>0.14445924666128415</v>
       </c>
       <c r="E10" s="0">
         <v>0.14445924666128415</v>
@@ -275,10 +474,10 @@
         <v>0.12028580961601032</v>
       </c>
       <c r="C11" s="0">
-        <v>0.28217701698753683</v>
+        <v>0.30067678194168734</v>
       </c>
       <c r="D11" s="0">
-        <v>0.27769117647058816</v>
+        <v>0.14705822437746419</v>
       </c>
       <c r="E11" s="0">
         <v>0.14705822437746419</v>
@@ -292,10 +491,10 @@
         <v>0.12335145444728568</v>
       </c>
       <c r="C12" s="0">
-        <v>0.28725217579576423</v>
+        <v>0.2970474802681361</v>
       </c>
       <c r="D12" s="0">
-        <v>0.28784117647058816</v>
+        <v>0.12118682526380609</v>
       </c>
       <c r="E12" s="0">
         <v>0.12118682526380609</v>
@@ -309,10 +508,10 @@
         <v>0.12253816368727177</v>
       </c>
       <c r="C13" s="0">
-        <v>0.28232056947125073</v>
+        <v>0.27622498188644162</v>
       </c>
       <c r="D13" s="0">
-        <v>0.2713411764705882</v>
+        <v>0.11721623604184339</v>
       </c>
       <c r="E13" s="0">
         <v>0.11721623604184339</v>
@@ -326,10 +525,10 @@
         <v>0.12394695234503317</v>
       </c>
       <c r="C14" s="0">
-        <v>0.28681770290508823</v>
+        <v>0.2446302972472974</v>
       </c>
       <c r="D14" s="0">
-        <v>0.32983333333333342</v>
+        <v>0.11447907527665702</v>
       </c>
       <c r="E14" s="0">
         <v>0.11447907527665702</v>
@@ -344,25 +543,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="13.453125" customWidth="true"/>
-    <col min="3" max="3" width="12.453125" customWidth="true"/>
-    <col min="4" max="4" width="12.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="13.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="12.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -376,10 +575,10 @@
         <v>0.080774699115163107</v>
       </c>
       <c r="C2" s="0">
-        <v>0.26439160324401634</v>
+        <v>0.98630281115949026</v>
       </c>
       <c r="D2" s="0">
-        <v>0.9040936672610117</v>
+        <v>0.36227338019890643</v>
       </c>
       <c r="E2" s="0">
         <v>0.36227338019890643</v>
@@ -393,10 +592,10 @@
         <v>0.34188220992921181</v>
       </c>
       <c r="C3" s="0">
-        <v>0.61150557584419007</v>
+        <v>0.45884907335200698</v>
       </c>
       <c r="D3" s="0">
-        <v>0.21675823510233472</v>
+        <v>0.82420010999812943</v>
       </c>
       <c r="E3" s="0">
         <v>0.82420010999812943</v>
@@ -410,10 +609,10 @@
         <v>0.38153112033192471</v>
       </c>
       <c r="C4" s="0">
-        <v>0.6744854014379118</v>
+        <v>0.30329144038982592</v>
       </c>
       <c r="D4" s="0">
-        <v>0.32710604680049049</v>
+        <v>0.89126168446223752</v>
       </c>
       <c r="E4" s="0">
         <v>0.89126168446223752</v>
@@ -427,10 +626,10 @@
         <v>0.3971616963747634</v>
       </c>
       <c r="C5" s="0">
-        <v>0.57214531405623759</v>
+        <v>0.1385319384612298</v>
       </c>
       <c r="D5" s="0">
-        <v>0.47013587950541857</v>
+        <v>0.28034418537177652</v>
       </c>
       <c r="E5" s="0">
         <v>0.28034418537177652</v>
@@ -444,10 +643,10 @@
         <v>0.57238004999006442</v>
       </c>
       <c r="C6" s="0">
-        <v>0.22215023384758981</v>
+        <v>0.21207200558351802</v>
       </c>
       <c r="D6" s="0">
-        <v>0.35230632758400404</v>
+        <v>0.25966657932140236</v>
       </c>
       <c r="E6" s="0">
         <v>0.25966657932140236</v>
@@ -461,10 +660,10 @@
         <v>0.57226936588887956</v>
       </c>
       <c r="C7" s="0">
-        <v>0.33341396415953672</v>
+        <v>0.22881227558070405</v>
       </c>
       <c r="D7" s="0">
-        <v>0.3693222414191859</v>
+        <v>0.18875763500450038</v>
       </c>
       <c r="E7" s="0">
         <v>0.18875763500450038</v>
@@ -478,10 +677,10 @@
         <v>0.62320385300580372</v>
       </c>
       <c r="C8" s="0">
-        <v>0.35184073484264156</v>
+        <v>0.22701581016204142</v>
       </c>
       <c r="D8" s="0">
-        <v>0.39997767636545611</v>
+        <v>0.38081537701960266</v>
       </c>
       <c r="E8" s="0">
         <v>0.38081537701960266</v>
@@ -495,10 +694,10 @@
         <v>0.77971250147684668</v>
       </c>
       <c r="C9" s="0">
-        <v>0.51952421044751618</v>
+        <v>0.44230089872626521</v>
       </c>
       <c r="D9" s="0">
-        <v>0.54963957526661544</v>
+        <v>0.56337910478406084</v>
       </c>
       <c r="E9" s="0">
         <v>0.56337910478406084</v>
@@ -512,10 +711,10 @@
         <v>0.7361592901476457</v>
       </c>
       <c r="C10" s="0">
-        <v>0.49609214301702098</v>
+        <v>0.3698206033043423</v>
       </c>
       <c r="D10" s="0">
-        <v>0.53125428291870436</v>
+        <v>0.58459165442681471</v>
       </c>
       <c r="E10" s="0">
         <v>0.58459165442681471</v>
@@ -529,10 +728,10 @@
         <v>0.61703138222671172</v>
       </c>
       <c r="C11" s="0">
-        <v>0.4027765824258096</v>
+        <v>0.39892763756255722</v>
       </c>
       <c r="D11" s="0">
-        <v>0.44151176286487315</v>
+        <v>0.69024857260347772</v>
       </c>
       <c r="E11" s="0">
         <v>0.69024857260347772</v>
@@ -546,10 +745,10 @@
         <v>0.72298359611422525</v>
       </c>
       <c r="C12" s="0">
-        <v>0.38251697542791807</v>
+        <v>0.36847947937082215</v>
       </c>
       <c r="D12" s="0">
-        <v>0.35973271618258429</v>
+        <v>0.69941477209038316</v>
       </c>
       <c r="E12" s="0">
         <v>0.69941477209038316</v>
@@ -563,10 +762,10 @@
         <v>0.6859995260339824</v>
       </c>
       <c r="C13" s="0">
-        <v>0.20644201946365104</v>
+        <v>0.32916211273864415</v>
       </c>
       <c r="D13" s="0">
-        <v>0.25612237502432222</v>
+        <v>0.72243648328844223</v>
       </c>
       <c r="E13" s="0">
         <v>0.72243648328844223</v>
@@ -580,10 +779,10 @@
         <v>0.64294299318384784</v>
       </c>
       <c r="C14" s="0">
-        <v>0.2389997533881546</v>
+        <v>0.44238210996018568</v>
       </c>
       <c r="D14" s="0">
-        <v>0.39363018367978364</v>
+        <v>0.65555132240198044</v>
       </c>
       <c r="E14" s="0">
         <v>0.65555132240198044</v>
@@ -598,25 +797,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="11.453125" customWidth="true"/>
-    <col min="3" max="3" width="11.453125" customWidth="true"/>
-    <col min="4" max="4" width="11.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>47</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -630,10 +829,10 @@
         <v>11.310373050058182</v>
       </c>
       <c r="C2" s="0">
-        <v>6.2686150368873008</v>
+        <v>2.1832080012246906</v>
       </c>
       <c r="D2" s="0">
-        <v>10.348805441666173</v>
+        <v>4.5359459429032647</v>
       </c>
       <c r="E2" s="0">
         <v>4.5359459429032647</v>
@@ -647,10 +846,10 @@
         <v>4.2063494686709362</v>
       </c>
       <c r="C3" s="0">
-        <v>2.8556627829275447</v>
+        <v>5.2730727287919308</v>
       </c>
       <c r="D3" s="0">
-        <v>6.0293477059913112</v>
+        <v>1.8335724740195507</v>
       </c>
       <c r="E3" s="0">
         <v>1.8335724740195507</v>
@@ -664,10 +863,10 @@
         <v>6.0864755704922846</v>
       </c>
       <c r="C4" s="0">
-        <v>3.6447777086518878</v>
+        <v>6.4716769795383975</v>
       </c>
       <c r="D4" s="0">
-        <v>6.0424680648604934</v>
+        <v>1.83337826894031</v>
       </c>
       <c r="E4" s="0">
         <v>1.83337826894031</v>
@@ -681,10 +880,10 @@
         <v>3.3361500232047177</v>
       </c>
       <c r="C5" s="0">
-        <v>7.4643060160823076</v>
+        <v>10.126771123626876</v>
       </c>
       <c r="D5" s="0">
-        <v>8.6748570781410681</v>
+        <v>7.0455390651760696</v>
       </c>
       <c r="E5" s="0">
         <v>7.0455390651760696</v>
@@ -698,10 +897,10 @@
         <v>3.5946592664624477</v>
       </c>
       <c r="C6" s="0">
-        <v>6.764498212686906</v>
+        <v>8.9286439084960456</v>
       </c>
       <c r="D6" s="0">
-        <v>7.8816824333534541</v>
+        <v>8.1879113709713387</v>
       </c>
       <c r="E6" s="0">
         <v>8.1879113709713387</v>
@@ -715,10 +914,10 @@
         <v>2.6893147151924195</v>
       </c>
       <c r="C7" s="0">
-        <v>6.5748053994505895</v>
+        <v>10.160678013519192</v>
       </c>
       <c r="D7" s="0">
-        <v>4.7782185172368239</v>
+        <v>8.3012145768689773</v>
       </c>
       <c r="E7" s="0">
         <v>8.3012145768689773</v>
@@ -732,10 +931,10 @@
         <v>1.6076729665983032</v>
       </c>
       <c r="C8" s="0">
-        <v>6.0890194058094513</v>
+        <v>5.2497130164138781</v>
       </c>
       <c r="D8" s="0">
-        <v>5.1773315060286542</v>
+        <v>4.582561459081572</v>
       </c>
       <c r="E8" s="0">
         <v>4.582561459081572</v>
@@ -749,10 +948,10 @@
         <v>1.7689752612794845</v>
       </c>
       <c r="C9" s="0">
-        <v>3.4811596166747729</v>
+        <v>4.6271382543123556</v>
       </c>
       <c r="D9" s="0">
-        <v>3.9100352601878074</v>
+        <v>2.7920475545336769</v>
       </c>
       <c r="E9" s="0">
         <v>2.7920475545336769</v>
@@ -766,10 +965,10 @@
         <v>2.6508436245070341</v>
       </c>
       <c r="C10" s="0">
-        <v>3.9222366359749783</v>
+        <v>4.6663087961106626</v>
       </c>
       <c r="D10" s="0">
-        <v>3.3555375570312065</v>
+        <v>2.3317895936403605</v>
       </c>
       <c r="E10" s="0">
         <v>2.3317895936403605</v>
@@ -783,10 +982,10 @@
         <v>3.6401267636416108</v>
       </c>
       <c r="C11" s="0">
-        <v>5.3343948012306157</v>
+        <v>6.9701224744067591</v>
       </c>
       <c r="D11" s="0">
-        <v>4.1697206940443383</v>
+        <v>3.1345067229620125</v>
       </c>
       <c r="E11" s="0">
         <v>3.1345067229620125</v>
@@ -800,10 +999,10 @@
         <v>5.0582584147927578</v>
       </c>
       <c r="C12" s="0">
-        <v>6.4848364612694382</v>
+        <v>5.5416378024277257</v>
       </c>
       <c r="D12" s="0">
-        <v>6.8909363122012977</v>
+        <v>4.8570547745804786</v>
       </c>
       <c r="E12" s="0">
         <v>4.8570547745804786</v>
@@ -817,10 +1016,10 @@
         <v>3.5704898994427943</v>
       </c>
       <c r="C13" s="0">
-        <v>10.166365925066453</v>
+        <v>5.0259223588549968</v>
       </c>
       <c r="D13" s="0">
-        <v>8.0946441573575605</v>
+        <v>7.6615030918961544</v>
       </c>
       <c r="E13" s="0">
         <v>7.6615030918961544</v>
@@ -834,10 +1033,10 @@
         <v>5.4818497585370025</v>
       </c>
       <c r="C14" s="0">
-        <v>10.849272887386421</v>
+        <v>4.4585884520124424</v>
       </c>
       <c r="D14" s="0">
-        <v>10.398368400260766</v>
+        <v>5.9239114981383159</v>
       </c>
       <c r="E14" s="0">
         <v>5.9239114981383159</v>
@@ -852,25 +1051,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="13.453125" customWidth="true"/>
-    <col min="3" max="3" width="13.453125" customWidth="true"/>
-    <col min="4" max="4" width="13.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="13.7109375" customWidth="true"/>
+    <col min="3" max="3" width="13.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="12.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -884,10 +1083,10 @@
         <v>0.04556187314083715</v>
       </c>
       <c r="C2" s="0">
-        <v>0.28095197937680649</v>
+        <v>0.82325773505948874</v>
       </c>
       <c r="D2" s="0">
-        <v>0.065934159812474857</v>
+        <v>0.47508844806562245</v>
       </c>
       <c r="E2" s="0">
         <v>0.47508844806562245</v>
@@ -901,10 +1100,10 @@
         <v>0.52010537443720994</v>
       </c>
       <c r="C3" s="0">
-        <v>0.72222660525769999</v>
+        <v>0.38347089093406117</v>
       </c>
       <c r="D3" s="0">
-        <v>0.30337372630887938</v>
+        <v>0.8716607140063426</v>
       </c>
       <c r="E3" s="0">
         <v>0.8716607140063426</v>
@@ -918,10 +1117,10 @@
         <v>0.29789519998872804</v>
       </c>
       <c r="C4" s="0">
-        <v>0.60160290372145275</v>
+        <v>0.26298783992291708</v>
       </c>
       <c r="D4" s="0">
-        <v>0.30210850133718625</v>
+        <v>0.87168634868618133</v>
       </c>
       <c r="E4" s="0">
         <v>0.87168634868618133</v>
@@ -935,10 +1134,10 @@
         <v>0.64831184081471371</v>
       </c>
       <c r="C5" s="0">
-        <v>0.18833496815765716</v>
+        <v>0.071721904219638533</v>
       </c>
       <c r="D5" s="0">
-        <v>0.12275722191961114</v>
+        <v>0.21727548313939571</v>
       </c>
       <c r="E5" s="0">
         <v>0.21727548313939571</v>
@@ -952,10 +1151,10 @@
         <v>0.60911535753991841</v>
       </c>
       <c r="C6" s="0">
-        <v>0.2387522589067097</v>
+        <v>0.11194438504131443</v>
       </c>
       <c r="D6" s="0">
-        <v>0.16287802013314512</v>
+        <v>0.14617901787395693</v>
       </c>
       <c r="E6" s="0">
         <v>0.14617901787395693</v>
@@ -969,10 +1168,10 @@
         <v>0.74775221307525874</v>
       </c>
       <c r="C7" s="0">
-        <v>0.2542306301362165</v>
+        <v>0.070808436062372082</v>
       </c>
       <c r="D7" s="0">
-        <v>0.44354192530370962</v>
+        <v>0.14039783457078692</v>
       </c>
       <c r="E7" s="0">
         <v>0.14039783457078692</v>
@@ -986,10 +1185,10 @@
         <v>0.90031990063735301</v>
       </c>
       <c r="C8" s="0">
-        <v>0.29765308304617999</v>
+        <v>0.38617118073176249</v>
       </c>
       <c r="D8" s="0">
-        <v>0.39462417095120983</v>
+        <v>0.46891356272249241</v>
       </c>
       <c r="E8" s="0">
         <v>0.46891356272249241</v>
@@ -1003,10 +1202,10 @@
         <v>0.88009802416272631</v>
       </c>
       <c r="C9" s="0">
-        <v>0.6262403163734791</v>
+        <v>0.46305502848960844</v>
       </c>
       <c r="D9" s="0">
-        <v>0.56244014060383152</v>
+        <v>0.73200815047061152</v>
       </c>
       <c r="E9" s="0">
         <v>0.73200815047061152</v>
@@ -1020,10 +1219,10 @@
         <v>0.7536258035205311</v>
       </c>
       <c r="C10" s="0">
-        <v>0.56066551840019718</v>
+        <v>0.45794475210120744</v>
       </c>
       <c r="D10" s="0">
-        <v>0.64535022834437294</v>
+        <v>0.80158674817841957</v>
       </c>
       <c r="E10" s="0">
         <v>0.80158674817841957</v>
@@ -1037,10 +1236,10 @@
         <v>0.60229868432803779</v>
       </c>
       <c r="C11" s="0">
-        <v>0.37644685644913833</v>
+        <v>0.22287183833508795</v>
       </c>
       <c r="D11" s="0">
-        <v>0.52524823579576074</v>
+        <v>0.67925773512266874</v>
       </c>
       <c r="E11" s="0">
         <v>0.67925773512266874</v>
@@ -1054,10 +1253,10 @@
         <v>0.40881174025499845</v>
       </c>
       <c r="C12" s="0">
-        <v>0.26185679626524494</v>
+        <v>0.35340174441808037</v>
       </c>
       <c r="D12" s="0">
-        <v>0.228878704627834</v>
+        <v>0.43357351053405857</v>
       </c>
       <c r="E12" s="0">
         <v>0.43357351053405857</v>
@@ -1071,10 +1270,10 @@
         <v>0.61274948032563126</v>
       </c>
       <c r="C13" s="0">
-        <v>0.070656266671980217</v>
+        <v>0.41272479065915291</v>
       </c>
       <c r="D13" s="0">
-        <v>0.15109616042044349</v>
+        <v>0.1759040293856704</v>
       </c>
       <c r="E13" s="0">
         <v>0.1759040293856704</v>
@@ -1088,10 +1287,10 @@
         <v>0.35994022587445329</v>
       </c>
       <c r="C14" s="0">
-        <v>0.054451726853882776</v>
+        <v>0.48544320784913431</v>
       </c>
       <c r="D14" s="0">
-        <v>0.064703186390835499</v>
+        <v>0.31369322259397492</v>
       </c>
       <c r="E14" s="0">
         <v>0.31369322259397492</v>
@@ -1106,25 +1305,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="12.453125" customWidth="true"/>
-    <col min="3" max="3" width="12.453125" customWidth="true"/>
-    <col min="4" max="4" width="11.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="12.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>55</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -1138,10 +1337,10 @@
         <v>0.23243697959960338</v>
       </c>
       <c r="C2" s="0">
-        <v>0.38279917192249074</v>
+        <v>0.42177813894609667</v>
       </c>
       <c r="D2" s="0">
-        <v>0.39695150802512702</v>
+        <v>0.14970635606411911</v>
       </c>
       <c r="E2" s="0">
         <v>0.14970635606411911</v>
@@ -1155,10 +1354,10 @@
         <v>0.42798625519345529</v>
       </c>
       <c r="C3" s="0">
-        <v>0.64530795270544239</v>
+        <v>0.66366945789004828</v>
       </c>
       <c r="D3" s="0">
-        <v>0.68666968698043562</v>
+        <v>0.38084778041425643</v>
       </c>
       <c r="E3" s="0">
         <v>0.38084778041425643</v>
@@ -1172,10 +1371,10 @@
         <v>0.64253225609436126</v>
       </c>
       <c r="C4" s="0">
-        <v>0.9786817028897028</v>
+        <v>0.9536298901713236</v>
       </c>
       <c r="D4" s="0">
-        <v>1.0100371677582949</v>
+        <v>0.65631106389548077</v>
       </c>
       <c r="E4" s="0">
         <v>0.65631106389548077</v>
@@ -1189,10 +1388,10 @@
         <v>0.93792708879238806</v>
       </c>
       <c r="C5" s="0">
-        <v>1.3303770236752275</v>
+        <v>1.2311483211392191</v>
       </c>
       <c r="D5" s="0">
-        <v>1.3534035651528424</v>
+        <v>0.99454338452565272</v>
       </c>
       <c r="E5" s="0">
         <v>0.99454338452565272</v>
@@ -1206,10 +1405,10 @@
         <v>1.2279973464570693</v>
       </c>
       <c r="C6" s="0">
-        <v>1.5381591136429245</v>
+        <v>1.4917149248518187</v>
       </c>
       <c r="D6" s="0">
-        <v>1.5506253769640745</v>
+        <v>1.3009648755745533</v>
       </c>
       <c r="E6" s="0">
         <v>1.3009648755745533</v>
@@ -1223,10 +1422,10 @@
         <v>1.3878356658437143</v>
       </c>
       <c r="C7" s="0">
-        <v>1.67210786318045</v>
+        <v>1.6149522587433645</v>
       </c>
       <c r="D7" s="0">
-        <v>1.6393887164094867</v>
+        <v>1.5206235019335639</v>
       </c>
       <c r="E7" s="0">
         <v>1.5206235019335639</v>
@@ -1240,10 +1439,10 @@
         <v>1.4865359190216194</v>
       </c>
       <c r="C8" s="0">
-        <v>1.6549083565420912</v>
+        <v>1.649643276309523</v>
       </c>
       <c r="D8" s="0">
-        <v>1.6314990170753816</v>
+        <v>1.7018521530192823</v>
       </c>
       <c r="E8" s="0">
         <v>1.7018521530192823</v>
@@ -1257,10 +1456,10 @@
         <v>1.4628481596506397</v>
       </c>
       <c r="C9" s="0">
-        <v>1.6127788988781362</v>
+        <v>1.6606673531671579</v>
       </c>
       <c r="D9" s="0">
-        <v>1.6022491283793574</v>
+        <v>1.7979209356956631</v>
       </c>
       <c r="E9" s="0">
         <v>1.7979209356956631</v>
@@ -1274,10 +1473,10 @@
         <v>1.4374174119017966</v>
       </c>
       <c r="C10" s="0">
-        <v>1.6221688004402059</v>
+        <v>1.6965747526409942</v>
       </c>
       <c r="D10" s="0">
-        <v>1.626322029380193</v>
+        <v>1.8622554958672355</v>
       </c>
       <c r="E10" s="0">
         <v>1.8622554958672355</v>
@@ -1291,10 +1490,10 @@
         <v>1.4238226186347196</v>
       </c>
       <c r="C11" s="0">
-        <v>1.6532518094309236</v>
+        <v>1.6930622802938313</v>
       </c>
       <c r="D11" s="0">
-        <v>1.6607035349915946</v>
+        <v>1.82501482774582</v>
       </c>
       <c r="E11" s="0">
         <v>1.82501482774582</v>
@@ -1308,10 +1507,10 @@
         <v>1.4286774206471711</v>
       </c>
       <c r="C12" s="0">
-        <v>1.6051795783926235</v>
+        <v>1.6925089605664392</v>
       </c>
       <c r="D12" s="0">
-        <v>1.6276203427245473</v>
+        <v>1.7613400328302078</v>
       </c>
       <c r="E12" s="0">
         <v>1.7613400328302078</v>
@@ -1325,10 +1524,10 @@
         <v>1.451296447746403</v>
       </c>
       <c r="C13" s="0">
-        <v>1.6375502202210743</v>
+        <v>1.6830872247684352</v>
       </c>
       <c r="D13" s="0">
-        <v>1.6518747142283592</v>
+        <v>1.6758990640002307</v>
       </c>
       <c r="E13" s="0">
         <v>1.6758990640002307</v>
@@ -1342,10 +1541,10 @@
         <v>1.4746662011956415</v>
       </c>
       <c r="C14" s="0">
-        <v>1.7088808411214109</v>
+        <v>1.6067678857926344</v>
       </c>
       <c r="D14" s="0">
-        <v>1.7079420804854182</v>
+        <v>1.5914571761222005</v>
       </c>
       <c r="E14" s="0">
         <v>1.5914571761222005</v>
@@ -1571,25 +1770,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="13.453125" customWidth="true"/>
-    <col min="3" max="3" width="12.453125" customWidth="true"/>
-    <col min="4" max="4" width="12.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="13.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
+    <col min="4" max="4" width="13.7109375" customWidth="true"/>
     <col min="5" max="5" width="13.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>58</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -1603,10 +1802,10 @@
         <v>0.075413994605982831</v>
       </c>
       <c r="C2" s="0">
-        <v>0.12473265465381604</v>
+        <v>0.14101289817245632</v>
       </c>
       <c r="D2" s="0">
-        <v>0.12999020642152023</v>
+        <v>0.047625892990788364</v>
       </c>
       <c r="E2" s="0">
         <v>0.047625892990788364</v>
@@ -1620,10 +1819,10 @@
         <v>0.13568801662487343</v>
       </c>
       <c r="C3" s="0">
-        <v>0.22823070126523168</v>
+        <v>0.22736368718657018</v>
       </c>
       <c r="D3" s="0">
-        <v>0.2452447834800256</v>
+        <v>0.1253054569698123</v>
       </c>
       <c r="E3" s="0">
         <v>0.1253054569698123</v>
@@ -1637,10 +1836,10 @@
         <v>0.21790256549684711</v>
       </c>
       <c r="C4" s="0">
-        <v>0.35697515206690739</v>
+        <v>0.33530784072201242</v>
       </c>
       <c r="D4" s="0">
-        <v>0.37028557078270818</v>
+        <v>0.22250796713553894</v>
       </c>
       <c r="E4" s="0">
         <v>0.22250796713553894</v>
@@ -1654,10 +1853,10 @@
         <v>0.3322978348547313</v>
       </c>
       <c r="C5" s="0">
-        <v>0.52297459341512942</v>
+        <v>0.44995290728094184</v>
       </c>
       <c r="D5" s="0">
-        <v>0.53059189430426601</v>
+        <v>0.34534841739864819</v>
       </c>
       <c r="E5" s="0">
         <v>0.34534841739864819</v>
@@ -1671,10 +1870,10 @@
         <v>0.45341381165739875</v>
       </c>
       <c r="C6" s="0">
-        <v>0.62236665075278552</v>
+        <v>0.58058833641054974</v>
       </c>
       <c r="D6" s="0">
-        <v>0.62628720846571939</v>
+        <v>0.45749946971555694</v>
       </c>
       <c r="E6" s="0">
         <v>0.45749946971555694</v>
@@ -1688,10 +1887,10 @@
         <v>0.52889127554226756</v>
       </c>
       <c r="C7" s="0">
-        <v>0.67885019603435781</v>
+        <v>0.62743580587985281</v>
       </c>
       <c r="D7" s="0">
-        <v>0.66648843882834996</v>
+        <v>0.53938743833695524</v>
       </c>
       <c r="E7" s="0">
         <v>0.53938743833695524</v>
@@ -1705,10 +1904,10 @@
         <v>0.57317274052486933</v>
       </c>
       <c r="C8" s="0">
-        <v>0.66195106670249826</v>
+        <v>0.64850958245241563</v>
       </c>
       <c r="D8" s="0">
-        <v>0.64674782728218039</v>
+        <v>0.61340724753053133</v>
       </c>
       <c r="E8" s="0">
         <v>0.61340724753053133</v>
@@ -1722,10 +1921,10 @@
         <v>0.56329457975912667</v>
       </c>
       <c r="C9" s="0">
-        <v>0.62502922143493078</v>
+        <v>0.6302297399039003</v>
       </c>
       <c r="D9" s="0">
-        <v>0.61808510398224337</v>
+        <v>0.65496684111559667</v>
       </c>
       <c r="E9" s="0">
         <v>0.65496684111559667</v>
@@ -1739,10 +1938,10 @@
         <v>0.55458147323792373</v>
       </c>
       <c r="C10" s="0">
-        <v>0.62810924114554811</v>
+        <v>0.62525069004960898</v>
       </c>
       <c r="D10" s="0">
-        <v>0.63215075956170907</v>
+        <v>0.68313739042265742</v>
       </c>
       <c r="E10" s="0">
         <v>0.68313739042265742</v>
@@ -1756,10 +1955,10 @@
         <v>0.55174103536397034</v>
       </c>
       <c r="C11" s="0">
-        <v>0.62877052606284978</v>
+        <v>0.61854347980070301</v>
       </c>
       <c r="D11" s="0">
-        <v>0.6325164264827785</v>
+        <v>0.67793205573863391</v>
       </c>
       <c r="E11" s="0">
         <v>0.67793205573863391</v>
@@ -1773,10 +1972,10 @@
         <v>0.55465746650519054</v>
       </c>
       <c r="C12" s="0">
-        <v>0.59576761389626198</v>
+        <v>0.61103455388735362</v>
       </c>
       <c r="D12" s="0">
-        <v>0.59634761263124847</v>
+        <v>0.66290070395606937</v>
       </c>
       <c r="E12" s="0">
         <v>0.66290070395606937</v>
@@ -1790,10 +1989,10 @@
         <v>0.56519091352602202</v>
       </c>
       <c r="C13" s="0">
-        <v>0.59620156251430123</v>
+        <v>0.60608462782483397</v>
       </c>
       <c r="D13" s="0">
-        <v>0.60611174636151788</v>
+        <v>0.63979298706644439</v>
       </c>
       <c r="E13" s="0">
         <v>0.63979298706644439</v>
@@ -1807,13 +2006,123 @@
         <v>0.57694591228644332</v>
       </c>
       <c r="C14" s="0">
-        <v>0.6388991366701825</v>
+        <v>0.59193648186500314</v>
       </c>
       <c r="D14" s="0">
-        <v>0.64617200310532852</v>
+        <v>0.61186566368660111</v>
       </c>
       <c r="E14" s="0">
         <v>0.61186566368660111</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="8.42578125" customWidth="true"/>
+    <col min="2" max="2" width="25.5703125" customWidth="true"/>
+    <col min="3" max="3" width="25.5703125" customWidth="true"/>
+    <col min="4" max="4" width="25.5703125" customWidth="true"/>
+    <col min="5" max="5" width="27.5703125" customWidth="true"/>
+    <col min="6" max="6" width="27.5703125" customWidth="true"/>
+    <col min="7" max="7" width="27.5703125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0</v>
+      </c>
+      <c r="C2" s="0">
+        <v>0.78700000000000003</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0</v>
+      </c>
+      <c r="E2" s="0">
+        <v>0</v>
+      </c>
+      <c r="F2" s="0">
+        <v>0</v>
+      </c>
+      <c r="G2" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0</v>
+      </c>
+      <c r="C3" s="0">
+        <v>0</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0</v>
+      </c>
+      <c r="E3" s="0">
+        <v>0</v>
+      </c>
+      <c r="F3" s="0">
+        <v>0</v>
+      </c>
+      <c r="G3" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0</v>
+      </c>
+      <c r="C4" s="0">
+        <v>0.99299999999999999</v>
+      </c>
+      <c r="D4" s="0">
+        <v>0</v>
+      </c>
+      <c r="E4" s="0">
+        <v>0</v>
+      </c>
+      <c r="F4" s="0">
+        <v>0</v>
+      </c>
+      <c r="G4" s="0">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1825,25 +2134,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="13.453125" customWidth="true"/>
-    <col min="3" max="3" width="15.453125" customWidth="true"/>
-    <col min="4" max="4" width="15.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="13.7109375" customWidth="true"/>
+    <col min="3" max="3" width="15.7109375" customWidth="true"/>
+    <col min="4" max="4" width="13.7109375" customWidth="true"/>
     <col min="5" max="5" width="13.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -1857,10 +2166,10 @@
         <v>0.057253154426277139</v>
       </c>
       <c r="C2" s="0">
-        <v>0.60114070888608317</v>
+        <v>0.88499436260551323</v>
       </c>
       <c r="D2" s="0">
-        <v>0.93365049339277917</v>
+        <v>0.42823522306298611</v>
       </c>
       <c r="E2" s="0">
         <v>0.42823522306298611</v>
@@ -1874,10 +2183,10 @@
         <v>0.22980440302497965</v>
       </c>
       <c r="C3" s="0">
-        <v>0.959338970652309</v>
+        <v>0.050364849876923141</v>
       </c>
       <c r="D3" s="0">
-        <v>0.8311310236204611</v>
+        <v>0.99660241506632852</v>
       </c>
       <c r="E3" s="0">
         <v>0.99660241506632852</v>
@@ -1891,10 +2200,10 @@
         <v>0.68520420611485233</v>
       </c>
       <c r="C4" s="0">
-        <v>0.57799726199262258</v>
+        <v>0.0094328683336404699</v>
       </c>
       <c r="D4" s="0">
-        <v>0.2316377679864404</v>
+        <v>0.82379311774893804</v>
       </c>
       <c r="E4" s="0">
         <v>0.82379311774893804</v>
@@ -1908,10 +2217,10 @@
         <v>0.7996992961152618</v>
       </c>
       <c r="C5" s="0">
-        <v>0.1003970796704793</v>
+        <v>0.012611417873592672</v>
       </c>
       <c r="D5" s="0">
-        <v>0.13079019621015342</v>
+        <v>0.15413821502129824</v>
       </c>
       <c r="E5" s="0">
         <v>0.15413821502129824</v>
@@ -1925,10 +2234,10 @@
         <v>0.38695838605692123</v>
       </c>
       <c r="C6" s="0">
-        <v>0.051670906991436685</v>
+        <v>0.013375942769567013</v>
       </c>
       <c r="D6" s="0">
-        <v>0.068254454174829032</v>
+        <v>0.08087228173322214</v>
       </c>
       <c r="E6" s="0">
         <v>0.08087228173322214</v>
@@ -1942,10 +2251,10 @@
         <v>0.19041557423737485</v>
       </c>
       <c r="C7" s="0">
-        <v>0.031438187963735743</v>
+        <v>0.023327637058906201</v>
       </c>
       <c r="D7" s="0">
-        <v>0.018665418998427694</v>
+        <v>0.12234717430472102</v>
       </c>
       <c r="E7" s="0">
         <v>0.12234717430472102</v>
@@ -1959,10 +2268,10 @@
         <v>0.20004818073291036</v>
       </c>
       <c r="C8" s="0">
-        <v>0.025083493037192452</v>
+        <v>0.046390262668114225</v>
       </c>
       <c r="D8" s="0">
-        <v>0.014751514480962168</v>
+        <v>0.21144946732769182</v>
       </c>
       <c r="E8" s="0">
         <v>0.21144946732769182</v>
@@ -1976,10 +2285,10 @@
         <v>0.34072796920471182</v>
       </c>
       <c r="C9" s="0">
-        <v>0.069277037602202038</v>
+        <v>0.00084757625997608206</v>
       </c>
       <c r="D9" s="0">
-        <v>0.068383633084909384</v>
+        <v>0.38371565443686895</v>
       </c>
       <c r="E9" s="0">
         <v>0.38371565443686895</v>
@@ -1993,10 +2302,10 @@
         <v>0.37118028876759912</v>
       </c>
       <c r="C10" s="0">
-        <v>0.00096829380931564668</v>
+        <v>0.0002500106218014344</v>
       </c>
       <c r="D10" s="0">
-        <v>0.0021253944487986754</v>
+        <v>0.21909716130549378</v>
       </c>
       <c r="E10" s="0">
         <v>0.21909716130549378</v>
@@ -2010,10 +2319,10 @@
         <v>0.42772236980564471</v>
       </c>
       <c r="C11" s="0">
-        <v>0.00043534004672940197</v>
+        <v>0.00013896121006472543</v>
       </c>
       <c r="D11" s="0">
-        <v>0.00056799041860469961</v>
+        <v>0.20226114807356005</v>
       </c>
       <c r="E11" s="0">
         <v>0.20226114807356005</v>
@@ -2027,10 +2336,10 @@
         <v>0.39604220917126903</v>
       </c>
       <c r="C12" s="0">
-        <v>0.00032055993293080541</v>
+        <v>0.0001748512954738456</v>
       </c>
       <c r="D12" s="0">
-        <v>0.00030926427435724874</v>
+        <v>0.41826360427005677</v>
       </c>
       <c r="E12" s="0">
         <v>0.41826360427005677</v>
@@ -2044,10 +2353,10 @@
         <v>0.40430680354021409</v>
       </c>
       <c r="C13" s="0">
-        <v>0.00043161995341552302</v>
+        <v>0.00061900590587613067</v>
       </c>
       <c r="D13" s="0">
-        <v>0.00082165899963096661</v>
+        <v>0.46082927443743044</v>
       </c>
       <c r="E13" s="0">
         <v>0.46082927443743044</v>
@@ -2061,10 +2370,10 @@
         <v>0.39005617847248836</v>
       </c>
       <c r="C14" s="0">
-        <v>0.00032914017960368594</v>
+        <v>0.0035365519162748678</v>
       </c>
       <c r="D14" s="0">
-        <v>1.9832031971538565e-05</v>
+        <v>0.49142986621215767</v>
       </c>
       <c r="E14" s="0">
         <v>0.49142986621215767</v>
@@ -2079,25 +2388,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="12.453125" customWidth="true"/>
-    <col min="3" max="3" width="12.453125" customWidth="true"/>
-    <col min="4" max="4" width="12.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" customWidth="true"/>
     <col min="5" max="5" width="12.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -2111,10 +2420,10 @@
         <v>1.4448535641802527</v>
       </c>
       <c r="C2" s="0">
-        <v>0.88516203509878677</v>
+        <v>0.57230666497361016</v>
       </c>
       <c r="D2" s="0">
-        <v>0.52268713046450921</v>
+        <v>0.8578292406658079</v>
       </c>
       <c r="E2" s="0">
         <v>0.8578292406658079</v>
@@ -2128,10 +2437,10 @@
         <v>1.0184619710257772</v>
       </c>
       <c r="C3" s="0">
-        <v>0.56137354720041832</v>
+        <v>1.3250097732048824</v>
       </c>
       <c r="D3" s="0">
-        <v>0.74723654934467643</v>
+        <v>0.53530226635665379</v>
       </c>
       <c r="E3" s="0">
         <v>0.53530226635665379</v>
@@ -2145,10 +2454,10 @@
         <v>0.84142956400602031</v>
       </c>
       <c r="C4" s="0">
-        <v>0.75816966711786837</v>
+        <v>1.6025427628320559</v>
       </c>
       <c r="D4" s="0">
-        <v>1.1572284658393641</v>
+        <v>0.75438512635022548</v>
       </c>
       <c r="E4" s="0">
         <v>0.75438512635022548</v>
@@ -2162,10 +2471,10 @@
         <v>0.76994379395053636</v>
       </c>
       <c r="C5" s="0">
-        <v>1.2001199278726546</v>
+        <v>1.5562872645608594</v>
       </c>
       <c r="D5" s="0">
-        <v>1.2825388157013304</v>
+        <v>1.1101319585086924</v>
       </c>
       <c r="E5" s="0">
         <v>1.1101319585086924</v>
@@ -2179,10 +2488,10 @@
         <v>1.0214055027339446</v>
       </c>
       <c r="C6" s="0">
-        <v>1.4629352589589928</v>
+        <v>1.6916897231365413</v>
       </c>
       <c r="D6" s="0">
-        <v>1.4086901746227725</v>
+        <v>1.2404883627275156</v>
       </c>
       <c r="E6" s="0">
         <v>1.2404883627275156</v>
@@ -2196,10 +2505,10 @@
         <v>1.2001199278726546</v>
       </c>
       <c r="C7" s="0">
-        <v>1.4128952199201537</v>
+        <v>1.6017017537725793</v>
       </c>
       <c r="D7" s="0">
-        <v>1.6374446388003217</v>
+        <v>1.1572284658393639</v>
       </c>
       <c r="E7" s="0">
         <v>1.1572284658393639</v>
@@ -2213,10 +2522,10 @@
         <v>1.1858227738615579</v>
       </c>
       <c r="C8" s="0">
-        <v>1.5916096450588633</v>
+        <v>1.4843809899756375</v>
       </c>
       <c r="D8" s="0">
-        <v>1.6559468381087992</v>
+        <v>1.0331796295666127</v>
       </c>
       <c r="E8" s="0">
         <v>1.0331796295666127</v>
@@ -2230,10 +2539,10 @@
         <v>1.0558868741724721</v>
       </c>
       <c r="C9" s="0">
-        <v>1.4057466429146055</v>
+        <v>1.9317978096170205</v>
       </c>
       <c r="D9" s="0">
-        <v>1.4095311836822486</v>
+        <v>0.9373045967863165</v>
       </c>
       <c r="E9" s="0">
         <v>0.9373045967863165</v>
@@ -2247,10 +2556,10 @@
         <v>1.0344411431558274</v>
       </c>
       <c r="C10" s="0">
-        <v>2.0545851323005575</v>
+        <v>2.0789743950253698</v>
       </c>
       <c r="D10" s="0">
-        <v>1.9545050542228797</v>
+        <v>1.0277130706800168</v>
       </c>
       <c r="E10" s="0">
         <v>1.0277130706800168</v>
@@ -2264,10 +2573,10 @@
         <v>0.99869825812808544</v>
       </c>
       <c r="C11" s="0">
-        <v>2.1529831922592826</v>
+        <v>2.1416295699563532</v>
       </c>
       <c r="D11" s="0">
-        <v>2.1172403072315409</v>
+        <v>1.0449537563992803</v>
       </c>
       <c r="E11" s="0">
         <v>1.0449537563992803</v>
@@ -2281,10 +2590,10 @@
         <v>1.0201439891447301</v>
       </c>
       <c r="C12" s="0">
-        <v>2.1887260772870247</v>
+        <v>2.1159787936423253</v>
       </c>
       <c r="D12" s="0">
-        <v>2.1887260772870247</v>
+        <v>0.99869825812808544</v>
       </c>
       <c r="E12" s="0">
         <v>0.99869825812808544</v>
@@ -2298,10 +2607,10 @@
         <v>1.0129954121391818</v>
       </c>
       <c r="C13" s="0">
-        <v>2.1555062194377115</v>
+        <v>1.9688022082339769</v>
       </c>
       <c r="D13" s="0">
-        <v>2.0743488451982492</v>
+        <v>0.97010395010589157</v>
       </c>
       <c r="E13" s="0">
         <v>0.97010395010589157</v>
@@ -2315,10 +2624,10 @@
         <v>1.0201439891447301</v>
       </c>
       <c r="C14" s="0">
-        <v>2.1849415365193812</v>
+        <v>1.7417297621753798</v>
       </c>
       <c r="D14" s="0">
-        <v>2.4919098432282243</v>
+        <v>0.95160175079741316</v>
       </c>
       <c r="E14" s="0">
         <v>0.95160175079741316</v>
@@ -2333,25 +2642,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="12.453125" customWidth="true"/>
-    <col min="3" max="3" width="12.453125" customWidth="true"/>
-    <col min="4" max="4" width="13.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="13.7109375" customWidth="true"/>
+    <col min="4" max="4" width="13.7109375" customWidth="true"/>
     <col min="5" max="5" width="13.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -2365,10 +2674,10 @@
         <v>0.66561602779249862</v>
       </c>
       <c r="C2" s="0">
-        <v>0.15693469940528762</v>
+        <v>0.039911499735029152</v>
       </c>
       <c r="D2" s="0">
-        <v>0.063506918683389257</v>
+        <v>0.11144191250073598</v>
       </c>
       <c r="E2" s="0">
         <v>0.11144191250073598</v>
@@ -2382,10 +2691,10 @@
         <v>0.27028552081493262</v>
       </c>
       <c r="C3" s="0">
-        <v>0.063209562503680136</v>
+        <v>0.35687534593416931</v>
       </c>
       <c r="D3" s="0">
-        <v>0.090138962491903674</v>
+        <v>0.039571983748454331</v>
       </c>
       <c r="E3" s="0">
         <v>0.039571983748454331</v>
@@ -2399,10 +2708,10 @@
         <v>0.17415020903256204</v>
       </c>
       <c r="C4" s="0">
-        <v>0.1514288406053112</v>
+        <v>0.64421562739209803</v>
       </c>
       <c r="D4" s="0">
-        <v>0.22873732556085488</v>
+        <v>0.061872696225637389</v>
       </c>
       <c r="E4" s="0">
         <v>0.061872696225637389</v>
@@ -2416,10 +2725,10 @@
         <v>0.10831861273037743</v>
       </c>
       <c r="C5" s="0">
-        <v>0.36194170641229467</v>
+        <v>0.84812977683565904</v>
       </c>
       <c r="D5" s="0">
-        <v>0.3830744862509568</v>
+        <v>0.27787605252311137</v>
       </c>
       <c r="E5" s="0">
         <v>0.27787605252311137</v>
@@ -2433,10 +2742,10 @@
         <v>0.17890184301949005</v>
       </c>
       <c r="C6" s="0">
-        <v>0.52927250780191959</v>
+        <v>0.84097656480009375</v>
       </c>
       <c r="D6" s="0">
-        <v>0.5563961019843372</v>
+        <v>0.47739934051698757</v>
       </c>
       <c r="E6" s="0">
         <v>0.47739934051698757</v>
@@ -2450,10 +2759,10 @@
         <v>0.23578808219984687</v>
       </c>
       <c r="C7" s="0">
-        <v>0.45528322440087143</v>
+        <v>0.73284737678855294</v>
       </c>
       <c r="D7" s="0">
-        <v>0.53013248542660307</v>
+        <v>0.39714408526173234</v>
       </c>
       <c r="E7" s="0">
         <v>0.39714408526173234</v>
@@ -2467,10 +2776,10 @@
         <v>0.2043972796325737</v>
       </c>
       <c r="C8" s="0">
-        <v>0.55379997644703527</v>
+        <v>0.69766007183654222</v>
       </c>
       <c r="D8" s="0">
-        <v>0.6936724371430254</v>
+        <v>0.2699519519519521</v>
       </c>
       <c r="E8" s="0">
         <v>0.2699519519519521</v>
@@ -2484,10 +2793,10 @@
         <v>0.16477112406524169</v>
       </c>
       <c r="C9" s="0">
-        <v>0.55018518518518511</v>
+        <v>0.87064111169993519</v>
       </c>
       <c r="D9" s="0">
-        <v>0.748033680739563</v>
+        <v>0.23832779838662185</v>
       </c>
       <c r="E9" s="0">
         <v>0.23832779838662185</v>
@@ -2501,10 +2810,10 @@
         <v>0.16482612023788482</v>
       </c>
       <c r="C10" s="0">
-        <v>1.0301260083613024</v>
+        <v>0.82976023081905437</v>
       </c>
       <c r="D10" s="0">
-        <v>1.1816833892716245</v>
+        <v>0.22932167461579223</v>
       </c>
       <c r="E10" s="0">
         <v>0.22932167461579223</v>
@@ -2518,10 +2827,10 @@
         <v>0.16616928693399274</v>
       </c>
       <c r="C11" s="0">
-        <v>1.3523262085615024</v>
+        <v>0.85330695401283663</v>
       </c>
       <c r="D11" s="0">
-        <v>1.5422494847788963</v>
+        <v>0.20642454218924802</v>
       </c>
       <c r="E11" s="0">
         <v>0.20642454218924802</v>
@@ -2535,10 +2844,10 @@
         <v>0.15394942000824352</v>
       </c>
       <c r="C12" s="0">
-        <v>1.5500850262026729</v>
+        <v>0.84626438202908771</v>
       </c>
       <c r="D12" s="0">
-        <v>1.68105134546311</v>
+        <v>0.17662862862862852</v>
       </c>
       <c r="E12" s="0">
         <v>0.17662862862862852</v>
@@ -2552,10 +2861,10 @@
         <v>0.16260813754931394</v>
       </c>
       <c r="C13" s="0">
-        <v>1.7792085026202675</v>
+        <v>0.84116151445563181</v>
       </c>
       <c r="D13" s="0">
-        <v>1.6743634811281867</v>
+        <v>0.15396019548960721</v>
       </c>
       <c r="E13" s="0">
         <v>0.15396019548960721</v>
@@ -2569,10 +2878,10 @@
         <v>0.15937154801860681</v>
       </c>
       <c r="C14" s="0">
-        <v>1.8205743979273388</v>
+        <v>0.80724736501207073</v>
       </c>
       <c r="D14" s="0">
-        <v>2.0048459047282572</v>
+        <v>0.16330389212742141</v>
       </c>
       <c r="E14" s="0">
         <v>0.16330389212742141</v>
@@ -2587,25 +2896,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="7.90625" customWidth="true"/>
-    <col min="3" max="3" width="11.453125" customWidth="true"/>
-    <col min="4" max="4" width="5.6328125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="8.42578125" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -2617,9 +2926,11 @@
       </c>
       <c r="B2" s="0"/>
       <c r="C2" s="0">
-        <v>40.252519476956223</v>
-      </c>
-      <c r="D2" s="0"/>
+        <v>23.499551735696116</v>
+      </c>
+      <c r="D2" s="0">
+        <v>4.102545020637649</v>
+      </c>
       <c r="E2" s="0">
         <v>4.102545020637649</v>
       </c>
@@ -2629,8 +2940,12 @@
         <v>1</v>
       </c>
       <c r="B3" s="0"/>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
+      <c r="C3" s="0">
+        <v>103.48152840608583</v>
+      </c>
+      <c r="D3" s="0">
+        <v>7.3539034012241302</v>
+      </c>
       <c r="E3" s="0">
         <v>7.3539034012241302</v>
       </c>
@@ -2640,10 +2955,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="0"/>
-      <c r="C4" s="0">
-        <v>143.67957300045822</v>
-      </c>
-      <c r="D4" s="0"/>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0">
+        <v>48.111820837812957</v>
+      </c>
       <c r="E4" s="0">
         <v>48.111820837812957</v>
       </c>
@@ -2654,9 +2969,11 @@
       </c>
       <c r="B5" s="0"/>
       <c r="C5" s="0">
-        <v>297.58821601247706</v>
-      </c>
-      <c r="D5" s="0"/>
+        <v>199.62836778252822</v>
+      </c>
+      <c r="D5" s="0">
+        <v>77.305199609286262</v>
+      </c>
       <c r="E5" s="0">
         <v>77.305199609286262</v>
       </c>
@@ -2667,7 +2984,9 @@
       </c>
       <c r="B6" s="0"/>
       <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
+      <c r="D6" s="0">
+        <v>107.95556365295391</v>
+      </c>
       <c r="E6" s="0">
         <v>107.95556365295391</v>
       </c>
@@ -2677,8 +2996,12 @@
         <v>5</v>
       </c>
       <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
+      <c r="C7" s="0">
+        <v>219.80793058546323</v>
+      </c>
+      <c r="D7" s="0">
+        <v>143.36114847978365</v>
+      </c>
       <c r="E7" s="0">
         <v>143.36114847978365</v>
       </c>
@@ -2688,8 +3011,12 @@
         <v>6</v>
       </c>
       <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
+      <c r="C8" s="0">
+        <v>251.67104090664512</v>
+      </c>
+      <c r="D8" s="0">
+        <v>154.45026491391332</v>
+      </c>
       <c r="E8" s="0">
         <v>154.45026491391332</v>
       </c>
@@ -2699,10 +3026,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="0"/>
-      <c r="C9" s="0">
-        <v>368.94720437398155</v>
-      </c>
-      <c r="D9" s="0"/>
+      <c r="C9" s="0"/>
+      <c r="D9" s="0">
+        <v>168.09663638751488</v>
+      </c>
       <c r="E9" s="0">
         <v>168.09663638751488</v>
       </c>
@@ -2713,9 +3040,11 @@
       </c>
       <c r="B10" s="0"/>
       <c r="C10" s="0">
-        <v>368.14730677816414</v>
-      </c>
-      <c r="D10" s="0"/>
+        <v>739.44211603886981</v>
+      </c>
+      <c r="D10" s="0">
+        <v>163.43768268987165</v>
+      </c>
       <c r="E10" s="0">
         <v>163.43768268987165</v>
       </c>
@@ -2726,9 +3055,11 @@
       </c>
       <c r="B11" s="0"/>
       <c r="C11" s="0">
-        <v>779.65610466692465</v>
-      </c>
-      <c r="D11" s="0"/>
+        <v>786.43418718487851</v>
+      </c>
+      <c r="D11" s="0">
+        <v>164.60306599042292</v>
+      </c>
       <c r="E11" s="0">
         <v>164.60306599042292</v>
       </c>
@@ -2739,9 +3070,11 @@
       </c>
       <c r="B12" s="0"/>
       <c r="C12" s="0">
-        <v>588.00153902104967</v>
-      </c>
-      <c r="D12" s="0"/>
+        <v>841.90295075722645</v>
+      </c>
+      <c r="D12" s="0">
+        <v>162.26112176095737</v>
+      </c>
       <c r="E12" s="0">
         <v>162.26112176095737</v>
       </c>
@@ -2752,9 +3085,11 @@
       </c>
       <c r="B13" s="0"/>
       <c r="C13" s="0">
-        <v>405.68210847490121</v>
-      </c>
-      <c r="D13" s="0"/>
+        <v>565.36760595288536</v>
+      </c>
+      <c r="D13" s="0">
+        <v>156.95342886341842</v>
+      </c>
       <c r="E13" s="0">
         <v>156.95342886341842</v>
       </c>
@@ -2765,7 +3100,9 @@
       </c>
       <c r="B14" s="0"/>
       <c r="C14" s="0"/>
-      <c r="D14" s="0"/>
+      <c r="D14" s="0">
+        <v>151.21155978980056</v>
+      </c>
       <c r="E14" s="0">
         <v>151.21155978980056</v>
       </c>
@@ -2779,25 +3116,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="7.90625" customWidth="true"/>
-    <col min="3" max="3" width="11.453125" customWidth="true"/>
-    <col min="4" max="4" width="5.6328125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="8.42578125" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -2809,9 +3146,11 @@
       </c>
       <c r="B2" s="0"/>
       <c r="C2" s="0">
-        <v>19.932739310572373</v>
-      </c>
-      <c r="D2" s="0"/>
+        <v>30.823336886142727</v>
+      </c>
+      <c r="D2" s="0">
+        <v>1.1525700710218132</v>
+      </c>
       <c r="E2" s="0">
         <v>1.1525700710218132</v>
       </c>
@@ -2821,8 +3160,12 @@
         <v>1</v>
       </c>
       <c r="B3" s="0"/>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
+      <c r="C3" s="0">
+        <v>22.645971418087697</v>
+      </c>
+      <c r="D3" s="0">
+        <v>7.0331928829762376</v>
+      </c>
       <c r="E3" s="0">
         <v>7.0331928829762376</v>
       </c>
@@ -2832,10 +3175,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="0"/>
-      <c r="C4" s="0">
-        <v>122.586574996661</v>
-      </c>
-      <c r="D4" s="0"/>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0">
+        <v>61.510459809574684</v>
+      </c>
       <c r="E4" s="0">
         <v>61.510459809574684</v>
       </c>
@@ -2846,9 +3189,11 @@
       </c>
       <c r="B5" s="0"/>
       <c r="C5" s="0">
-        <v>135.2195184912743</v>
-      </c>
-      <c r="D5" s="0"/>
+        <v>57.174486635840253</v>
+      </c>
+      <c r="D5" s="0">
+        <v>84.562793947282159</v>
+      </c>
       <c r="E5" s="0">
         <v>84.562793947282159</v>
       </c>
@@ -2859,7 +3204,9 @@
       </c>
       <c r="B6" s="0"/>
       <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
+      <c r="D6" s="0">
+        <v>109.82543981605426</v>
+      </c>
       <c r="E6" s="0">
         <v>109.82543981605426</v>
       </c>
@@ -2869,8 +3216,12 @@
         <v>5</v>
       </c>
       <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
+      <c r="C7" s="0">
+        <v>90.78634365075726</v>
+      </c>
+      <c r="D7" s="0">
+        <v>182.31115007559163</v>
+      </c>
       <c r="E7" s="0">
         <v>182.31115007559163</v>
       </c>
@@ -2880,8 +3231,12 @@
         <v>6</v>
       </c>
       <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
+      <c r="C8" s="0">
+        <v>202.39035591627672</v>
+      </c>
+      <c r="D8" s="0">
+        <v>182.34643895422647</v>
+      </c>
       <c r="E8" s="0">
         <v>182.34643895422647</v>
       </c>
@@ -2891,10 +3246,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="0"/>
-      <c r="C9" s="0">
-        <v>240.26874047158893</v>
-      </c>
-      <c r="D9" s="0"/>
+      <c r="C9" s="0"/>
+      <c r="D9" s="0">
+        <v>256.37795289458921</v>
+      </c>
       <c r="E9" s="0">
         <v>256.37795289458921</v>
       </c>
@@ -2905,9 +3260,11 @@
       </c>
       <c r="B10" s="0"/>
       <c r="C10" s="0">
-        <v>208.16219916669496</v>
-      </c>
-      <c r="D10" s="0"/>
+        <v>168.05236176556426</v>
+      </c>
+      <c r="D10" s="0">
+        <v>263.67317777309006</v>
+      </c>
       <c r="E10" s="0">
         <v>263.67317777309006</v>
       </c>
@@ -2918,9 +3275,11 @@
       </c>
       <c r="B11" s="0"/>
       <c r="C11" s="0">
-        <v>241.19554100870147</v>
-      </c>
-      <c r="D11" s="0"/>
+        <v>273.9730323327808</v>
+      </c>
+      <c r="D11" s="0">
+        <v>336.16436167684458</v>
+      </c>
       <c r="E11" s="0">
         <v>336.16436167684458</v>
       </c>
@@ -2931,9 +3290,11 @@
       </c>
       <c r="B12" s="0"/>
       <c r="C12" s="0">
-        <v>351.47693973091151</v>
-      </c>
-      <c r="D12" s="0"/>
+        <v>185.65833742080852</v>
+      </c>
+      <c r="D12" s="0">
+        <v>384.99781655124912</v>
+      </c>
       <c r="E12" s="0">
         <v>384.99781655124912</v>
       </c>
@@ -2944,9 +3305,11 @@
       </c>
       <c r="B13" s="0"/>
       <c r="C13" s="0">
-        <v>329.91677438183217</v>
-      </c>
-      <c r="D13" s="0"/>
+        <v>183.22946468266829</v>
+      </c>
+      <c r="D13" s="0">
+        <v>404.5340559007588</v>
+      </c>
       <c r="E13" s="0">
         <v>404.5340559007588</v>
       </c>
@@ -2957,7 +3320,9 @@
       </c>
       <c r="B14" s="0"/>
       <c r="C14" s="0"/>
-      <c r="D14" s="0"/>
+      <c r="D14" s="0">
+        <v>413.76260622931738</v>
+      </c>
       <c r="E14" s="0">
         <v>413.76260622931738</v>
       </c>
@@ -2971,25 +3336,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="7.90625" customWidth="true"/>
-    <col min="3" max="3" width="16.08984375" customWidth="true"/>
-    <col min="4" max="4" width="5.6328125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="8.42578125" customWidth="true"/>
+    <col min="3" max="3" width="16.5703125" customWidth="true"/>
+    <col min="4" max="4" width="15.5703125" customWidth="true"/>
     <col min="5" max="5" width="15.08984375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -3001,9 +3366,11 @@
       </c>
       <c r="B2" s="0"/>
       <c r="C2" s="0">
-        <v>9.419465653997908e-09</v>
-      </c>
-      <c r="D2" s="0"/>
+        <v>3.1771009842324958e-05</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0.2506019020623938</v>
+      </c>
       <c r="E2" s="0">
         <v>0.2506019020623938</v>
       </c>
@@ -3013,8 +3380,12 @@
         <v>1</v>
       </c>
       <c r="B3" s="0"/>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
+      <c r="C3" s="0">
+        <v>2.7719201801933043e-22</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0.061433545629179569</v>
+      </c>
       <c r="E3" s="0">
         <v>0.061433545629179569</v>
       </c>
@@ -3024,10 +3395,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="0"/>
-      <c r="C4" s="0">
-        <v>6.08144014261919e-31</v>
-      </c>
-      <c r="D4" s="0"/>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0">
+        <v>2.0159401300893981e-10</v>
+      </c>
       <c r="E4" s="0">
         <v>2.0159401300893981e-10</v>
       </c>
@@ -3038,9 +3409,11 @@
       </c>
       <c r="B5" s="0"/>
       <c r="C5" s="0">
-        <v>3.3093292244312381e-64</v>
-      </c>
-      <c r="D5" s="0"/>
+        <v>5.0752952181669581e-43</v>
+      </c>
+      <c r="D5" s="0">
+        <v>1.1613052047621201e-16</v>
+      </c>
       <c r="E5" s="0">
         <v>1.1613052047621201e-16</v>
       </c>
@@ -3051,7 +3424,9 @@
       </c>
       <c r="B6" s="0"/>
       <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
+      <c r="D6" s="0">
+        <v>3.021887021613542e-23</v>
+      </c>
       <c r="E6" s="0">
         <v>3.021887021613542e-23</v>
       </c>
@@ -3061,8 +3436,12 @@
         <v>5</v>
       </c>
       <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
+      <c r="C7" s="0">
+        <v>2.209217911592923e-47</v>
+      </c>
+      <c r="D7" s="0">
+        <v>7.1232180943007404e-31</v>
+      </c>
       <c r="E7" s="0">
         <v>7.1232180943007404e-31</v>
       </c>
@@ -3072,8 +3451,12 @@
         <v>6</v>
       </c>
       <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
+      <c r="C8" s="0">
+        <v>2.8470821477862339e-54</v>
+      </c>
+      <c r="D8" s="0">
+        <v>2.8884879520704878e-33</v>
+      </c>
       <c r="E8" s="0">
         <v>2.8884879520704878e-33</v>
       </c>
@@ -3083,10 +3466,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="0"/>
-      <c r="C9" s="0">
-        <v>1.1768661089676433e-79</v>
-      </c>
-      <c r="D9" s="0"/>
+      <c r="C9" s="0"/>
+      <c r="D9" s="0">
+        <v>3.2776282916285198e-36</v>
+      </c>
       <c r="E9" s="0">
         <v>3.2776282916285198e-36</v>
       </c>
@@ -3097,9 +3480,11 @@
       </c>
       <c r="B10" s="0"/>
       <c r="C10" s="0">
-        <v>1.7536941418629181e-79</v>
-      </c>
-      <c r="D10" s="0"/>
+        <v>5.8770982633450092e-160</v>
+      </c>
+      <c r="D10" s="0">
+        <v>3.3205312805652342e-35</v>
+      </c>
       <c r="E10" s="0">
         <v>3.3205312805652342e-35</v>
       </c>
@@ -3110,9 +3495,11 @@
       </c>
       <c r="B11" s="0"/>
       <c r="C11" s="0">
-        <v>1.1175720957153711e-168</v>
-      </c>
-      <c r="D11" s="0"/>
+        <v>3.7871150553915377e-170</v>
+      </c>
+      <c r="D11" s="0">
+        <v>1.8606821516641195e-35</v>
+      </c>
       <c r="E11" s="0">
         <v>1.8606821516641195e-35</v>
       </c>
@@ -3123,9 +3510,11 @@
       </c>
       <c r="B12" s="0"/>
       <c r="C12" s="0">
-        <v>4.0221118006367018e-127</v>
-      </c>
-      <c r="D12" s="0"/>
+        <v>3.5333210767465764e-182</v>
+      </c>
+      <c r="D12" s="0">
+        <v>5.958604994619762e-35</v>
+      </c>
       <c r="E12" s="0">
         <v>5.958604994619762e-35</v>
       </c>
@@ -3136,9 +3525,11 @@
       </c>
       <c r="B13" s="0"/>
       <c r="C13" s="0">
-        <v>1.3012149032406678e-87</v>
-      </c>
-      <c r="D13" s="0"/>
+        <v>3.2423201937087272e-122</v>
+      </c>
+      <c r="D13" s="0">
+        <v>8.328417465922568e-34</v>
+      </c>
       <c r="E13" s="0">
         <v>8.328417465922568e-34</v>
       </c>
@@ -3149,7 +3540,9 @@
       </c>
       <c r="B14" s="0"/>
       <c r="C14" s="0"/>
-      <c r="D14" s="0"/>
+      <c r="D14" s="0">
+        <v>1.4434564514749968e-32</v>
+      </c>
       <c r="E14" s="0">
         <v>1.4434564514749968e-32</v>
       </c>
@@ -3163,25 +3556,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="7.90625" customWidth="true"/>
-    <col min="3" max="3" width="15.08984375" customWidth="true"/>
-    <col min="4" max="4" width="5.6328125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="8.42578125" customWidth="true"/>
+    <col min="3" max="3" width="15.5703125" customWidth="true"/>
+    <col min="4" max="4" width="15.5703125" customWidth="true"/>
     <col min="5" max="5" width="15.08984375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -3193,9 +3586,11 @@
       </c>
       <c r="B2" s="0"/>
       <c r="C2" s="0">
-        <v>8.0214861321270696e-06</v>
-      </c>
-      <c r="D2" s="0"/>
+        <v>2.8261862505246383e-08</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0.28301178936396537</v>
+      </c>
       <c r="E2" s="0">
         <v>0.28301178936396537</v>
       </c>
@@ -3205,8 +3600,12 @@
         <v>1</v>
       </c>
       <c r="B3" s="0"/>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
+      <c r="C3" s="0">
+        <v>1.9476816385331773e-06</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0.0080012570667795501</v>
+      </c>
       <c r="E3" s="0">
         <v>0.0080012570667795501</v>
       </c>
@@ -3216,10 +3615,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="0"/>
-      <c r="C4" s="0">
-        <v>1.7175477143039229e-28</v>
-      </c>
-      <c r="D4" s="0"/>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0">
+        <v>4.4039737637122979e-15</v>
+      </c>
       <c r="E4" s="0">
         <v>4.4039737637122979e-15</v>
       </c>
@@ -3230,9 +3629,11 @@
       </c>
       <c r="B5" s="0"/>
       <c r="C5" s="0">
-        <v>2.9561097497409038e-31</v>
-      </c>
-      <c r="D5" s="0"/>
+        <v>3.9881136845624667e-14</v>
+      </c>
+      <c r="D5" s="0">
+        <v>3.722038797096414e-20</v>
+      </c>
       <c r="E5" s="0">
         <v>3.722038797096414e-20</v>
       </c>
@@ -3243,7 +3644,9 @@
       </c>
       <c r="B6" s="0"/>
       <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
+      <c r="D6" s="0">
+        <v>1.0701117979021874e-25</v>
+      </c>
       <c r="E6" s="0">
         <v>1.0701117979021874e-25</v>
       </c>
@@ -3253,8 +3656,12 @@
         <v>5</v>
       </c>
       <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
+      <c r="C7" s="0">
+        <v>1.6005422573396206e-21</v>
+      </c>
+      <c r="D7" s="0">
+        <v>1.516421268160008e-41</v>
+      </c>
       <c r="E7" s="0">
         <v>1.516421268160008e-41</v>
       </c>
@@ -3264,8 +3671,12 @@
         <v>6</v>
       </c>
       <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
+      <c r="C8" s="0">
+        <v>6.2837345120133246e-46</v>
+      </c>
+      <c r="D8" s="0">
+        <v>1.4897568989231308e-41</v>
+      </c>
       <c r="E8" s="0">
         <v>1.4897568989231308e-41</v>
       </c>
@@ -3275,10 +3686,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="0"/>
-      <c r="C9" s="0">
-        <v>3.4364358516261076e-54</v>
-      </c>
-      <c r="D9" s="0"/>
+      <c r="C9" s="0"/>
+      <c r="D9" s="0">
+        <v>1.0569558793742522e-57</v>
+      </c>
       <c r="E9" s="0">
         <v>1.0569558793742522e-57</v>
       </c>
@@ -3289,9 +3700,11 @@
       </c>
       <c r="B10" s="0"/>
       <c r="C10" s="0">
-        <v>3.4580404034259217e-47</v>
-      </c>
-      <c r="D10" s="0"/>
+        <v>1.9704441934260533e-38</v>
+      </c>
+      <c r="D10" s="0">
+        <v>2.7156403742695119e-59</v>
+      </c>
       <c r="E10" s="0">
         <v>2.7156403742695119e-59</v>
       </c>
@@ -3302,9 +3715,11 @@
       </c>
       <c r="B11" s="0"/>
       <c r="C11" s="0">
-        <v>2.1578778929215194e-54</v>
-      </c>
-      <c r="D11" s="0"/>
+        <v>1.5453509570086629e-61</v>
+      </c>
+      <c r="D11" s="0">
+        <v>4.3673514368927565e-75</v>
+      </c>
       <c r="E11" s="0">
         <v>4.3673514368927565e-75</v>
       </c>
@@ -3315,9 +3730,11 @@
       </c>
       <c r="B12" s="0"/>
       <c r="C12" s="0">
-        <v>2.020770360454294e-78</v>
-      </c>
-      <c r="D12" s="0"/>
+        <v>2.8188929377822207e-42</v>
+      </c>
+      <c r="D12" s="0">
+        <v>1.0159596986109038e-85</v>
+      </c>
       <c r="E12" s="0">
         <v>1.0159596986109038e-85</v>
       </c>
@@ -3328,9 +3745,11 @@
       </c>
       <c r="B13" s="0"/>
       <c r="C13" s="0">
-        <v>1.002106814076956e-73</v>
-      </c>
-      <c r="D13" s="0"/>
+        <v>9.5572064505263673e-42</v>
+      </c>
+      <c r="D13" s="0">
+        <v>5.6746802464205869e-90</v>
+      </c>
       <c r="E13" s="0">
         <v>5.6746802464205869e-90</v>
       </c>
@@ -3341,7 +3760,9 @@
       </c>
       <c r="B14" s="0"/>
       <c r="C14" s="0"/>
-      <c r="D14" s="0"/>
+      <c r="D14" s="0">
+        <v>5.5604857959076311e-92</v>
+      </c>
       <c r="E14" s="0">
         <v>5.5604857959076311e-92</v>
       </c>
@@ -3355,25 +3776,25 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" customWidth="true"/>
-    <col min="2" max="2" width="11.453125" customWidth="true"/>
-    <col min="3" max="3" width="11.453125" customWidth="true"/>
-    <col min="4" max="4" width="11.453125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.453125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="E1" s="0" t="s">
         <v>3</v>
@@ -3387,10 +3808,10 @@
         <v>8.3126266983605959</v>
       </c>
       <c r="C2" s="0">
-        <v>5.2311495347686714</v>
+        <v>0.35080503951792413</v>
       </c>
       <c r="D2" s="0">
-        <v>1.0372654016798095</v>
+        <v>4.3373344470204183</v>
       </c>
       <c r="E2" s="0">
         <v>4.3373344470204183</v>
@@ -3404,10 +3825,10 @@
         <v>4.5056149602957341</v>
       </c>
       <c r="C3" s="0">
-        <v>2.6869188673537829</v>
+        <v>3.6268858120984033</v>
       </c>
       <c r="D3" s="0">
-        <v>5.7729506668559871</v>
+        <v>1.5137666630525857</v>
       </c>
       <c r="E3" s="0">
         <v>1.5137666630525857</v>
@@ -3421,10 +3842,10 @@
         <v>4.1851261623299312</v>
       </c>
       <c r="C4" s="0">
-        <v>2.3345532126631072</v>
+        <v>4.8476342736765865</v>
       </c>
       <c r="D4" s="0">
-        <v>4.6326588784777201</v>
+        <v>1.1189021861390649</v>
       </c>
       <c r="E4" s="0">
         <v>1.1189021861390649</v>
@@ -3438,10 +3859,10 @@
         <v>4.0658926264673276</v>
       </c>
       <c r="C5" s="0">
-        <v>2.9150230906927028</v>
+        <v>6.9504139612940676</v>
       </c>
       <c r="D5" s="0">
-        <v>3.5512014405528793</v>
+        <v>5.0684673943504732</v>
       </c>
       <c r="E5" s="0">
         <v>5.0684673943504732</v>
@@ -3455,10 +3876,10 @@
         <v>2.9136397165325798</v>
       </c>
       <c r="C6" s="0">
-        <v>5.7066845959689658</v>
+        <v>5.8317317810756233</v>
       </c>
       <c r="D6" s="0">
-        <v>4.4186205629752733</v>
+        <v>5.280939041366036</v>
       </c>
       <c r="E6" s="0">
         <v>5.280939041366036</v>
@@ -3472,10 +3893,10 @@
         <v>2.9142919760446864</v>
       </c>
       <c r="C7" s="0">
-        <v>4.5778677860671753</v>
+        <v>5.626731003970904</v>
       </c>
       <c r="D7" s="0">
-        <v>4.2809053840235256</v>
+        <v>6.1424775149568287</v>
       </c>
       <c r="E7" s="0">
         <v>6.1424775149568287</v>
@@ -3489,10 +3910,10 @@
         <v>2.6204553750818151</v>
       </c>
       <c r="C8" s="0">
-        <v>4.422462047437965</v>
+        <v>5.648088316952629</v>
       </c>
       <c r="D8" s="0">
-        <v>4.0447933056541823</v>
+        <v>4.190675127316986</v>
       </c>
       <c r="E8" s="0">
         <v>4.190675127316986</v>
@@ -3506,10 +3927,10 @@
         <v>1.7604349006010982</v>
       </c>
       <c r="C9" s="0">
-        <v>3.2335807831589238</v>
+        <v>3.740236018664203</v>
       </c>
       <c r="D9" s="0">
-        <v>3.0491177591468879</v>
+        <v>2.966904133106059</v>
       </c>
       <c r="E9" s="0">
         <v>2.966904133106059</v>
@@ -3523,10 +3944,10 @@
         <v>1.9978231570506517</v>
       </c>
       <c r="C10" s="0">
-        <v>3.3817023111533735</v>
+        <v>4.2769478279583284</v>
       </c>
       <c r="D10" s="0">
-        <v>3.1609924092545936</v>
+        <v>2.8420762587298061</v>
       </c>
       <c r="E10" s="0">
         <v>2.8420762587298061</v>
@@ -3540,10 +3961,10 @@
         <v>2.6554562746202</v>
       </c>
       <c r="C11" s="0">
-        <v>4.0239328338367679</v>
+        <v>4.0526477601697461</v>
       </c>
       <c r="D11" s="0">
-        <v>3.7457159062015828</v>
+        <v>2.2480173831133943</v>
       </c>
       <c r="E11" s="0">
         <v>2.2480173831133943</v>
@@ -3557,10 +3978,10 @@
         <v>2.0694673846627882</v>
       </c>
       <c r="C12" s="0">
-        <v>4.1774962286332418</v>
+        <v>4.2876073766891238</v>
       </c>
       <c r="D12" s="0">
-        <v>4.3578852119919205</v>
+        <v>2.197894473236826</v>
       </c>
       <c r="E12" s="0">
         <v>2.197894473236826</v>
@@ -3574,10 +3995,10 @@
         <v>2.2712977138599477</v>
       </c>
       <c r="C13" s="0">
-        <v>5.9038861074403739</v>
+        <v>4.6147062214987162</v>
       </c>
       <c r="D13" s="0">
-        <v>5.3187975804830092</v>
+        <v>2.072443627961492</v>
       </c>
       <c r="E13" s="0">
         <v>2.072443627961492</v>
@@ -3591,10 +4012,10 @@
         <v>2.5094580165031122</v>
       </c>
       <c r="C14" s="0">
-        <v>5.5083126866546674</v>
+        <v>3.7396724711257185</v>
       </c>
       <c r="D14" s="0">
-        <v>4.0925141620532104</v>
+        <v>2.4392206863846564</v>
       </c>
       <c r="E14" s="0">
         <v>2.4392206863846564</v>

</xml_diff>